<commit_message>
feat: add PCIe slot compatibility validation for card configuration
Implement PCIe card-to-slot compatibility checking in the server
configurator. Adds slot type definitions per product (pcieSlots column
in products.xlsx) and interface type per card (pcie_interface column in
config_options.xlsx).

Compatibility rules:
- PCIe x16 double width slots accept x16 double width, x16, and x8 cards
- PCIe x16 slots accept x16 and x8 cards (backward compatible)
- OCP3.0 slots only accept NIC cards; only GPU uses double width
- 1U chassis: RAID BBU reserves one additional PCIe x8 slot
- Greedy slot assignment prioritizes most restrictive cards first

Includes visual slot usage panel on config page and blocks submission
when slot capacity is exceeded. Product slot layouts use placeholder
data to be updated with real values.

https://claude.ai/code/session_01XmZdxA3cNiZ5ah4jR4MqVu
</commit_message>
<xml_diff>
--- a/config_options.xlsx
+++ b/config_options.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>qty_editable</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pcie_interface</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -509,6 +514,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -556,6 +562,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,6 +610,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -650,6 +658,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -697,6 +706,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -744,6 +754,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -791,6 +802,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -838,6 +850,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -885,6 +898,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -932,6 +946,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -979,6 +994,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1026,6 +1042,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1073,6 +1090,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1120,6 +1138,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1167,6 +1186,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1214,6 +1234,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1261,6 +1282,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1308,6 +1330,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1355,6 +1378,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1402,6 +1426,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1449,6 +1474,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1496,6 +1522,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1543,6 +1570,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1590,6 +1618,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1637,6 +1666,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1684,6 +1714,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1731,6 +1762,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1778,6 +1810,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1825,6 +1858,7 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1872,6 +1906,7 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1919,6 +1954,7 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1966,6 +2002,7 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2013,6 +2050,7 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2060,6 +2098,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2107,6 +2146,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2154,6 +2198,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2201,6 +2250,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>PCIe x16</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2248,6 +2302,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>PCIe x16</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2295,6 +2354,11 @@
           <t>true</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2342,6 +2406,7 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2389,6 +2454,11 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2436,6 +2506,11 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2483,6 +2558,11 @@
           <t>false</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>PCIe x8</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2528,6 +2608,11 @@
       <c r="I45" t="inlineStr">
         <is>
           <t>false</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>PCIe x16</t>
         </is>
       </c>
     </row>

</xml_diff>